<commit_message>
Restore /us/en/ URL structure to match wknd.site source
- Point all content import scripts at /us/en/... output paths
  (home -> /us/en, hub + leaf pages under /us/en/magazine and
  /us/en/adventures, about-us, faqs, search)
- Rewrite nav/footer internal links + brand link to /us/en targets
- Keep /us/en prefix in link-rewrite transformers (was being stripped)
- Narrow publish/preview scripts to the canonical /us/en tree + global
  nav/footer; drop stale bare-path duplicates
- Add redirects sheet mapping / and legacy bare paths to /us/en twins

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-wknd-about-us.report.xlsx
+++ b/tools/importer/reports/import-wknd-about-us.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="199">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,7 +73,7 @@
     <t>adventures.report.json</t>
   </si>
   <si>
-    <t>["teaser-columns","cards-magazine"]</t>
+    <t>["teaser-columns","cards-adventures"]</t>
   </si>
   <si>
     <t>adventures</t>
@@ -82,7 +82,7 @@
     <t>wknd-adventures</t>
   </si>
   <si>
-    <t>2026-08-11T06:01:51.714Z</t>
+    <t>2026-08-11T06:35:24.757Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -145,7 +145,7 @@
     <t>wknd-faqs</t>
   </si>
   <si>
-    <t>2026-08-11T06:01:46.477Z</t>
+    <t>2026-08-11T06:03:25.152Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -163,7 +163,7 @@
     <t>wknd-footer</t>
   </si>
   <si>
-    <t>2026-08-10T10:18:15.420Z</t>
+    <t>2026-08-12T10:41:01.214Z</t>
   </si>
   <si>
     <t>Footer</t>
@@ -184,7 +184,7 @@
     <t>wknd-home</t>
   </si>
   <si>
-    <t>2026-08-11T06:03:09.258Z</t>
+    <t>2026-08-11T06:06:15.138Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -196,7 +196,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-08-11T06:01:40.639Z</t>
+    <t>2026-08-11T06:22:12.226Z</t>
   </si>
   <si>
     <t>nav.report.json</t>
@@ -511,7 +511,7 @@
     <t>magazine/arctic-surfing</t>
   </si>
   <si>
-    <t>2026-08-07T09:09:26.685Z</t>
+    <t>2026-08-11T06:19:20.905Z</t>
   </si>
   <si>
     <t>magazine/guide-la-skateparks.report.json</t>
@@ -520,7 +520,7 @@
     <t>magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-08-07T09:09:31.643Z</t>
+    <t>2026-08-11T06:19:26.676Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -535,7 +535,7 @@
     <t>magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-08-07T09:09:35.685Z</t>
+    <t>2026-08-11T06:19:33.009Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -550,7 +550,7 @@
     <t>magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-08-07T09:09:39.945Z</t>
+    <t>2026-08-11T06:19:38.359Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -565,13 +565,31 @@
     <t>magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-08-07T09:09:44.331Z</t>
+    <t>2026-08-11T06:19:43.878Z</t>
   </si>
   <si>
     <t>Western Australia</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/western-australia.html</t>
+  </si>
+  <si>
+    <t>us/en.report.json</t>
+  </si>
+  <si>
+    <t>us/en</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:10:23.761Z</t>
+  </si>
+  <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:10:28.532Z</t>
   </si>
   <si>
     <t>us/en/adventures/yosemite-backpacking.html.report.json</t>
@@ -980,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
@@ -2083,30 +2101,94 @@
         <v>187</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="C35" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
         <v>188</v>
       </c>
-      <c r="D35" t="s">
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>56</v>
+      </c>
+      <c r="H35" t="s">
         <v>189</v>
       </c>
-      <c r="E35" t="s">
+      <c r="I35" t="s">
+        <v>58</v>
+      </c>
+      <c r="J35" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>190</v>
       </c>
-      <c r="F35" t="s">
+      <c r="B36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
         <v>191</v>
       </c>
-      <c r="G35" t="s">
-        <v>12</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
         <v>192</v>
       </c>
-      <c r="I35" t="s">
-        <v>12</v>
-      </c>
-      <c r="J35" t="s">
+      <c r="I36" t="s">
+        <v>17</v>
+      </c>
+      <c r="J36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>193</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>194</v>
+      </c>
+      <c r="D37" t="s">
+        <v>195</v>
+      </c>
+      <c r="E37" t="s">
+        <v>196</v>
+      </c>
+      <c r="F37" t="s">
+        <v>197</v>
+      </c>
+      <c r="G37" t="s">
+        <v>12</v>
+      </c>
+      <c r="H37" t="s">
+        <v>198</v>
+      </c>
+      <c r="I37" t="s">
+        <v>12</v>
+      </c>
+      <c r="J37" t="s">
         <v>153</v>
       </c>
     </row>

</xml_diff>